<commit_message>
feat: read excel value as string
</commit_message>
<xml_diff>
--- a/e1.xlsx
+++ b/e1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\excel-compare\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5E56B9E-0E67-4074-919B-A9548984A118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A456425-B079-432E-8074-A8E98DC32554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="13546" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
   <si>
     <t>系统名称</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -187,23 +187,35 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ABC</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>BBC</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>S5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>S6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CDC</t>
+    <t>50000012345001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50000012345001.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50000012345002</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50000012345003</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>S4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -281,11 +293,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -778,6 +791,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14C1ED27-6622-4C3F-9A5F-289FFE36F446}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="3" max="3" width="26.6640625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="16.86328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
@@ -786,7 +803,7 @@
       <c r="B1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>33</v>
       </c>
       <c r="D1" t="s">
@@ -800,11 +817,11 @@
       <c r="B2" t="s">
         <v>35</v>
       </c>
-      <c r="C2">
-        <v>100</v>
-      </c>
-      <c r="D2">
-        <v>99</v>
+      <c r="C2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
@@ -812,13 +829,13 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3">
-        <v>99</v>
-      </c>
-      <c r="D3">
-        <v>100</v>
+        <v>48</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
@@ -828,50 +845,53 @@
       <c r="B4" t="s">
         <v>37</v>
       </c>
-      <c r="C4">
-        <v>10.1</v>
-      </c>
-      <c r="D4">
-        <v>1.1000000000000001</v>
+      <c r="C4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C5">
-        <v>10.1</v>
-      </c>
-      <c r="D5">
-        <v>1.1000000000000001</v>
+        <v>35</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="B6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6">
-        <v>10.1</v>
-      </c>
-      <c r="D6">
-        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
         <v>37</v>
       </c>
-      <c r="D7">
-        <v>3</v>
+      <c r="C7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>